<commit_message>
Change contact person in all invoice templates
</commit_message>
<xml_diff>
--- a/cg/apps/invoice/templates/KI_pool_invoice.xlsx
+++ b/cg/apps/invoice/templates/KI_pool_invoice.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10107"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10404"/>
   <workbookPr autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/christian/Documents/clinicalGenomics/cg/cg/apps/invoice/templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/linnealofdahl/dev/cg/cg/apps/invoice/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CC3DEF9-34E1-6F4D-927E-B7F554680798}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E97E1AD-7EA9-7C4E-82B5-94E4DAA24393}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="18000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Faktura" sheetId="1" r:id="rId1"/>
@@ -118,13 +118,13 @@
     <t>Total</t>
   </si>
   <si>
-    <t>Anna Zetterlund</t>
+    <t>Anna Gellerbring</t>
   </si>
   <si>
-    <t>anna.zetterlund@scilifelab.se</t>
+    <t>anna.gellerbring@scilifelab.se</t>
   </si>
   <si>
-    <t>(+46) 701523463</t>
+    <t>(+46) 701904409</t>
   </si>
 </sst>
 </file>
@@ -346,6 +346,9 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -357,9 +360,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -593,10 +593,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="31"/>
+      <c r="B1" s="32"/>
       <c r="C1" s="4" t="s">
         <v>1</v>
       </c>
@@ -629,10 +629,10 @@
       <c r="Z1" s="7"/>
     </row>
     <row r="2" spans="1:26" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="32" t="s">
+      <c r="A2" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="31"/>
+      <c r="B2" s="32"/>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
       <c r="E2" s="5" t="s">
@@ -881,7 +881,7 @@
         <v>15</v>
       </c>
       <c r="B10" s="5"/>
-      <c r="C10" s="35" t="s">
+      <c r="C10" s="30" t="s">
         <v>32</v>
       </c>
       <c r="D10" s="5"/>
@@ -35650,10 +35650,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="31"/>
+      <c r="B1" s="32"/>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
@@ -35666,10 +35666,10 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="35" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="31"/>
+      <c r="B2" s="32"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="3" t="s">

</xml_diff>

<commit_message>
Change contact person in all invoice templates (#5019)
### Changed

- Switched from AZ to AG as contact person in invoicing templates
</commit_message>
<xml_diff>
--- a/cg/apps/invoice/templates/KI_pool_invoice.xlsx
+++ b/cg/apps/invoice/templates/KI_pool_invoice.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10107"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10404"/>
   <workbookPr autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/christian/Documents/clinicalGenomics/cg/cg/apps/invoice/templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/linnealofdahl/dev/cg/cg/apps/invoice/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CC3DEF9-34E1-6F4D-927E-B7F554680798}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E97E1AD-7EA9-7C4E-82B5-94E4DAA24393}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="18000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Faktura" sheetId="1" r:id="rId1"/>
@@ -118,13 +118,13 @@
     <t>Total</t>
   </si>
   <si>
-    <t>Anna Zetterlund</t>
+    <t>Anna Gellerbring</t>
   </si>
   <si>
-    <t>anna.zetterlund@scilifelab.se</t>
+    <t>anna.gellerbring@scilifelab.se</t>
   </si>
   <si>
-    <t>(+46) 701523463</t>
+    <t>(+46) 701904409</t>
   </si>
 </sst>
 </file>
@@ -346,6 +346,9 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -357,9 +360,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -593,10 +593,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="31"/>
+      <c r="B1" s="32"/>
       <c r="C1" s="4" t="s">
         <v>1</v>
       </c>
@@ -629,10 +629,10 @@
       <c r="Z1" s="7"/>
     </row>
     <row r="2" spans="1:26" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="32" t="s">
+      <c r="A2" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="31"/>
+      <c r="B2" s="32"/>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
       <c r="E2" s="5" t="s">
@@ -881,7 +881,7 @@
         <v>15</v>
       </c>
       <c r="B10" s="5"/>
-      <c r="C10" s="35" t="s">
+      <c r="C10" s="30" t="s">
         <v>32</v>
       </c>
       <c r="D10" s="5"/>
@@ -35650,10 +35650,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="31"/>
+      <c r="B1" s="32"/>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
@@ -35666,10 +35666,10 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="35" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="31"/>
+      <c r="B2" s="32"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="3" t="s">

</xml_diff>